<commit_message>
problemas con subir al drive y los  hilos
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BISAGRA T.xlsx
+++ b/LISTAS/ma/BISAGRA T.xlsx
@@ -743,17 +743,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="17" t="n">
-        <v>45163.60824765425</v>
+        <v>45232</v>
       </c>
       <c r="E1" s="13" t="n"/>
       <c r="F1" s="13" t="n"/>
       <c r="G1" s="13" t="n"/>
     </row>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
     <row r="7" ht="22.5" customHeight="1" s="14">
       <c r="A7" s="23" t="inlineStr">
         <is>
@@ -792,14 +787,6 @@
     <row r="12" ht="33.75" customHeight="1" s="14">
       <c r="A12" s="6" t="n"/>
     </row>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21" ht="18" customHeight="1" s="14">
       <c r="A21" s="18" t="inlineStr">
         <is>
@@ -831,7 +818,7 @@
       </c>
       <c r="C22" s="22" t="n"/>
       <c r="D22" s="11" t="n">
-        <v>4928.755</v>
+        <v>5668.068</v>
       </c>
       <c r="H22" s="9" t="n"/>
     </row>
@@ -848,7 +835,7 @@
       </c>
       <c r="C23" s="22" t="n"/>
       <c r="D23" s="11" t="n">
-        <v>5583.487</v>
+        <v>6421.01</v>
       </c>
       <c r="H23" s="9" t="n"/>
     </row>
@@ -865,7 +852,7 @@
       </c>
       <c r="C24" s="22" t="n"/>
       <c r="D24" s="11" t="n">
-        <v>7273.126</v>
+        <v>8364.094999999999</v>
       </c>
       <c r="H24" s="9" t="n"/>
     </row>
@@ -882,14 +869,10 @@
       </c>
       <c r="C25" s="22" t="n"/>
       <c r="D25" s="12" t="n">
-        <v>8056.975</v>
+        <v>9265.521000000001</v>
       </c>
       <c r="H25" s="9" t="n"/>
     </row>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
     <row r="30" ht="18.75" customHeight="1" s="14">
       <c r="A30" s="7" t="inlineStr">
         <is>
@@ -904,21 +887,6 @@
         </is>
       </c>
     </row>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
     <row r="47" ht="15" customHeight="1" s="14">
       <c r="A47" s="8" t="inlineStr">
         <is>
@@ -928,12 +896,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B21:C21"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B25:C25"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B22:C22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>